<commit_message>
Phase 2 complete: live draft pick grid (Q6)
Encode the confirmed card-draw pick order and build the draft-day tool.

- draft/order.py: DRAFT_ORDER (slot -> pick per round), 121-pick sequence,
  slot picks, picks-until-next; validated (each round a permutation of 1-11)
- board payload gains the draft order + sequence + roster template
- web "Draft Room" mode: set the card # you drew, then click each player as
  taken. Tracks on-the-clock slot, your next pick and picks-until, your roster
  filling (C/K/DEF/QB/RB×3/R×4), best-available-for-need recommendation, and a
  "⚠ likely gone before your pick" at-risk line (top-N available by VOR, where
  N = picks until your next turn). Undo + localStorage persistence.
- tests: draft-order validity + helpers (145 total)

Our draft slot is drawn on the day; the tool works for any slot immediately.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Fantasy Football Schedule.xlsx
+++ b/Fantasy Football Schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/8d7edda75b0035ba/Documents/Projects/Fantasy Football/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{5137DF5C-90EF-4497-8F7C-12860CB6FCAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DBA56FC3-40A5-4C3C-AD2D-6FBB47F6FA72}"/>
+  <xr:revisionPtr revIDLastSave="169" documentId="8_{5137DF5C-90EF-4497-8F7C-12860CB6FCAD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{DA4A2478-68FC-4470-994F-53089A5F51FC}"/>
   <bookViews>
-    <workbookView xWindow="-57720" yWindow="45" windowWidth="29040" windowHeight="15720" xr2:uid="{96F0BD3F-329E-4C7B-9E0C-1D36DD946968}"/>
+    <workbookView xWindow="-49125" yWindow="3195" windowWidth="16200" windowHeight="9990" xr2:uid="{96F0BD3F-329E-4C7B-9E0C-1D36DD946968}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="188" uniqueCount="157">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="170">
   <si>
     <t>Sept 18 - Sept 22</t>
   </si>
@@ -510,13 +510,63 @@
   </si>
   <si>
     <t>R10 - B3</t>
+  </si>
+  <si>
+    <t>Round</t>
+  </si>
+  <si>
+    <t>Ace Spades</t>
+  </si>
+  <si>
+    <t>2 Spades</t>
+  </si>
+  <si>
+    <t>3 Spades</t>
+  </si>
+  <si>
+    <t>4 Spades</t>
+  </si>
+  <si>
+    <t>5 Spades</t>
+  </si>
+  <si>
+    <t>6 Spades</t>
+  </si>
+  <si>
+    <t>7 Spades</t>
+  </si>
+  <si>
+    <t>8 Spades</t>
+  </si>
+  <si>
+    <t>9 Spades</t>
+  </si>
+  <si>
+    <t>10 Spades</t>
+  </si>
+  <si>
+    <t>Jack Spades</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Draft Pick Slot based on Card Drawn - </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>for example, who ever draws the 4 Spades will have pick #4 in the First Round, pick #8 Second Round, pick #5 Third Round, etc.</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -569,6 +619,19 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="7">
     <fill>
@@ -608,7 +671,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="7">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -638,51 +701,11 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom/>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right/>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top/>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="4" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -691,55 +714,32 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="0" fontId="3" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="4" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="5" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1079,718 +1079,1179 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{26BE20EF-F4EF-4587-9100-0AD92A4BB0B7}">
-  <dimension ref="A1:S25"/>
+  <dimension ref="A1:S33"/>
   <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="17.46484375" customWidth="1"/>
     <col min="2" max="24" width="15.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A1" s="16" t="s">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A1" s="11" t="s">
         <v>43</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="D1" s="18" t="s">
+      <c r="B1" s="12"/>
+      <c r="C1" s="8" t="s">
         <v>44</v>
       </c>
-      <c r="E1" s="19"/>
-    </row>
-    <row r="2" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A2" s="20" t="s">
+      <c r="E1" s="16" t="s">
+        <v>169</v>
+      </c>
+    </row>
+    <row r="2" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A2" s="11" t="s">
         <v>45</v>
       </c>
-      <c r="B2" s="21"/>
-      <c r="D2" s="22" t="s">
+      <c r="B2" s="12"/>
+      <c r="C2" s="13" t="s">
         <v>45</v>
       </c>
-      <c r="E2" s="23"/>
-    </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A3" s="6">
+      <c r="E2" s="15" t="s">
+        <v>157</v>
+      </c>
+      <c r="F2">
         <v>1</v>
       </c>
-      <c r="B3" s="7">
+      <c r="G2">
+        <v>2</v>
+      </c>
+      <c r="H2">
+        <v>3</v>
+      </c>
+      <c r="I2">
+        <v>4</v>
+      </c>
+      <c r="J2">
+        <v>5</v>
+      </c>
+      <c r="K2">
+        <v>6</v>
+      </c>
+      <c r="L2">
         <v>7</v>
       </c>
-      <c r="C3" s="5"/>
-      <c r="D3" s="10">
+      <c r="M2">
+        <v>8</v>
+      </c>
+      <c r="N2">
+        <v>9</v>
+      </c>
+      <c r="O2">
+        <v>10</v>
+      </c>
+      <c r="P2">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="3" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A3" s="9">
         <v>1</v>
       </c>
-      <c r="E3" s="11">
+      <c r="B3" s="9"/>
+      <c r="C3" s="10">
+        <v>1</v>
+      </c>
+      <c r="E3" s="14" t="s">
+        <v>158</v>
+      </c>
+      <c r="F3">
+        <v>1</v>
+      </c>
+      <c r="G3">
+        <v>11</v>
+      </c>
+      <c r="H3">
+        <v>8</v>
+      </c>
+      <c r="I3">
+        <v>4</v>
+      </c>
+      <c r="J3">
+        <v>1</v>
+      </c>
+      <c r="K3">
+        <v>11</v>
+      </c>
+      <c r="L3">
+        <v>8</v>
+      </c>
+      <c r="M3">
+        <v>4</v>
+      </c>
+      <c r="N3">
+        <v>1</v>
+      </c>
+      <c r="O3">
+        <v>11</v>
+      </c>
+      <c r="P3">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="4" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A4" s="9">
+        <v>2</v>
+      </c>
+      <c r="B4" s="9"/>
+      <c r="C4" s="10">
+        <v>2</v>
+      </c>
+      <c r="E4" s="14" t="s">
+        <v>159</v>
+      </c>
+      <c r="F4">
+        <v>2</v>
+      </c>
+      <c r="G4">
+        <v>10</v>
+      </c>
+      <c r="H4">
         <v>7</v>
       </c>
-    </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A4" s="6">
+      <c r="I4">
+        <v>5</v>
+      </c>
+      <c r="J4">
         <v>2</v>
       </c>
-      <c r="B4" s="7">
+      <c r="K4">
+        <v>10</v>
+      </c>
+      <c r="L4">
+        <v>7</v>
+      </c>
+      <c r="M4">
+        <v>5</v>
+      </c>
+      <c r="N4">
+        <v>2</v>
+      </c>
+      <c r="O4">
+        <v>10</v>
+      </c>
+      <c r="P4">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A5" s="9">
+        <v>3</v>
+      </c>
+      <c r="B5" s="9"/>
+      <c r="C5" s="10">
+        <v>3</v>
+      </c>
+      <c r="E5" s="14" t="s">
+        <v>160</v>
+      </c>
+      <c r="F5">
+        <v>3</v>
+      </c>
+      <c r="G5">
+        <v>9</v>
+      </c>
+      <c r="H5">
+        <v>6</v>
+      </c>
+      <c r="I5">
+        <v>6</v>
+      </c>
+      <c r="J5">
+        <v>3</v>
+      </c>
+      <c r="K5">
+        <v>9</v>
+      </c>
+      <c r="L5">
+        <v>6</v>
+      </c>
+      <c r="M5">
+        <v>6</v>
+      </c>
+      <c r="N5">
+        <v>3</v>
+      </c>
+      <c r="O5">
+        <v>9</v>
+      </c>
+      <c r="P5">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="6" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A6" s="9">
+        <v>4</v>
+      </c>
+      <c r="B6" s="9"/>
+      <c r="C6" s="10">
+        <v>4</v>
+      </c>
+      <c r="E6" s="14" t="s">
+        <v>161</v>
+      </c>
+      <c r="F6">
+        <v>4</v>
+      </c>
+      <c r="G6">
         <v>8</v>
       </c>
-      <c r="C4" s="5"/>
-      <c r="D4" s="10">
+      <c r="H6">
+        <v>5</v>
+      </c>
+      <c r="I6">
+        <v>7</v>
+      </c>
+      <c r="J6">
+        <v>4</v>
+      </c>
+      <c r="K6">
+        <v>8</v>
+      </c>
+      <c r="L6">
+        <v>5</v>
+      </c>
+      <c r="M6">
+        <v>7</v>
+      </c>
+      <c r="N6">
+        <v>4</v>
+      </c>
+      <c r="O6">
+        <v>8</v>
+      </c>
+      <c r="P6">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A7" s="9">
+        <v>5</v>
+      </c>
+      <c r="B7" s="9"/>
+      <c r="C7" s="10">
+        <v>5</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>162</v>
+      </c>
+      <c r="F7">
+        <v>5</v>
+      </c>
+      <c r="G7">
+        <v>7</v>
+      </c>
+      <c r="H7">
+        <v>1</v>
+      </c>
+      <c r="I7">
+        <v>11</v>
+      </c>
+      <c r="J7">
+        <v>5</v>
+      </c>
+      <c r="K7">
+        <v>7</v>
+      </c>
+      <c r="L7">
+        <v>1</v>
+      </c>
+      <c r="M7">
+        <v>11</v>
+      </c>
+      <c r="N7">
+        <v>5</v>
+      </c>
+      <c r="O7">
+        <v>7</v>
+      </c>
+      <c r="P7">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="8" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A8" s="9">
+        <v>6</v>
+      </c>
+      <c r="B8" s="9"/>
+      <c r="C8" s="10">
+        <v>6</v>
+      </c>
+      <c r="E8" s="14" t="s">
+        <v>163</v>
+      </c>
+      <c r="F8">
+        <v>6</v>
+      </c>
+      <c r="G8">
+        <v>6</v>
+      </c>
+      <c r="H8">
         <v>2</v>
       </c>
-      <c r="E4" s="11">
+      <c r="I8">
+        <v>10</v>
+      </c>
+      <c r="J8">
+        <v>6</v>
+      </c>
+      <c r="K8">
+        <v>6</v>
+      </c>
+      <c r="L8">
+        <v>2</v>
+      </c>
+      <c r="M8">
+        <v>10</v>
+      </c>
+      <c r="N8">
+        <v>6</v>
+      </c>
+      <c r="O8">
+        <v>6</v>
+      </c>
+      <c r="P8">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="9" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A9" s="9">
+        <v>7</v>
+      </c>
+      <c r="B9" s="9"/>
+      <c r="C9" s="10">
+        <v>7</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>164</v>
+      </c>
+      <c r="F9">
+        <v>7</v>
+      </c>
+      <c r="G9">
+        <v>5</v>
+      </c>
+      <c r="H9">
+        <v>3</v>
+      </c>
+      <c r="I9">
+        <v>9</v>
+      </c>
+      <c r="J9">
+        <v>7</v>
+      </c>
+      <c r="K9">
+        <v>5</v>
+      </c>
+      <c r="L9">
+        <v>3</v>
+      </c>
+      <c r="M9">
+        <v>9</v>
+      </c>
+      <c r="N9">
+        <v>7</v>
+      </c>
+      <c r="O9">
+        <v>5</v>
+      </c>
+      <c r="P9">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A10" s="9">
         <v>8</v>
       </c>
-    </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A5" s="6">
+      <c r="B10" s="9"/>
+      <c r="C10" s="10">
+        <v>8</v>
+      </c>
+      <c r="E10" s="14" t="s">
+        <v>165</v>
+      </c>
+      <c r="F10">
+        <v>8</v>
+      </c>
+      <c r="G10">
+        <v>4</v>
+      </c>
+      <c r="H10">
+        <v>4</v>
+      </c>
+      <c r="I10">
+        <v>8</v>
+      </c>
+      <c r="J10">
+        <v>8</v>
+      </c>
+      <c r="K10">
+        <v>4</v>
+      </c>
+      <c r="L10">
+        <v>4</v>
+      </c>
+      <c r="M10">
+        <v>8</v>
+      </c>
+      <c r="N10">
+        <v>8</v>
+      </c>
+      <c r="O10">
+        <v>4</v>
+      </c>
+      <c r="P10">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="11" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A11" s="9">
+        <v>9</v>
+      </c>
+      <c r="B11" s="9"/>
+      <c r="C11" s="10">
+        <v>9</v>
+      </c>
+      <c r="E11" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="F11">
+        <v>9</v>
+      </c>
+      <c r="G11">
         <v>3</v>
       </c>
-      <c r="B5" s="7">
+      <c r="H11">
+        <v>11</v>
+      </c>
+      <c r="I11">
+        <v>1</v>
+      </c>
+      <c r="J11">
         <v>9</v>
       </c>
-      <c r="C5" s="5"/>
-      <c r="D5" s="10">
+      <c r="K11">
         <v>3</v>
       </c>
-      <c r="E5" s="11">
+      <c r="L11">
+        <v>11</v>
+      </c>
+      <c r="M11">
+        <v>1</v>
+      </c>
+      <c r="N11">
         <v>9</v>
       </c>
-    </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A6" s="6">
+      <c r="O11">
+        <v>3</v>
+      </c>
+      <c r="P11">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="12" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A12" s="9">
+        <v>10</v>
+      </c>
+      <c r="B12" s="9"/>
+      <c r="C12" s="10">
+        <v>10</v>
+      </c>
+      <c r="E12" s="14" t="s">
+        <v>167</v>
+      </c>
+      <c r="F12">
+        <v>10</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+      <c r="H12">
+        <v>10</v>
+      </c>
+      <c r="I12">
+        <v>2</v>
+      </c>
+      <c r="J12">
+        <v>10</v>
+      </c>
+      <c r="K12">
+        <v>2</v>
+      </c>
+      <c r="L12">
+        <v>10</v>
+      </c>
+      <c r="M12">
+        <v>2</v>
+      </c>
+      <c r="N12">
+        <v>10</v>
+      </c>
+      <c r="O12">
+        <v>2</v>
+      </c>
+      <c r="P12">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A13" s="9">
+        <v>11</v>
+      </c>
+      <c r="B13" s="9"/>
+      <c r="C13" s="10">
+        <v>11</v>
+      </c>
+      <c r="E13" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="F13">
+        <v>11</v>
+      </c>
+      <c r="G13">
+        <v>1</v>
+      </c>
+      <c r="H13">
+        <v>9</v>
+      </c>
+      <c r="I13">
+        <v>3</v>
+      </c>
+      <c r="J13">
+        <v>11</v>
+      </c>
+      <c r="K13">
+        <v>1</v>
+      </c>
+      <c r="L13">
+        <v>9</v>
+      </c>
+      <c r="M13">
+        <v>3</v>
+      </c>
+      <c r="N13">
+        <v>11</v>
+      </c>
+      <c r="O13">
+        <v>1</v>
+      </c>
+      <c r="P13">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="14" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A14" s="9"/>
+      <c r="B14" s="9"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="10"/>
+      <c r="E14" s="10"/>
+    </row>
+    <row r="15" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A15" s="9"/>
+      <c r="B15" s="9"/>
+      <c r="C15" s="5"/>
+      <c r="D15" s="10"/>
+      <c r="E15" s="10"/>
+    </row>
+    <row r="16" spans="1:16" x14ac:dyDescent="0.45">
+      <c r="A16" s="9"/>
+      <c r="B16" s="9"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="10"/>
+      <c r="E16" s="10"/>
+    </row>
+    <row r="17" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A17" s="5"/>
+    </row>
+    <row r="18" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A18" s="7" t="s">
+        <v>155</v>
+      </c>
+    </row>
+    <row r="19" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A19" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="D19" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E19" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="G19" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="H19" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I19" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="J19" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="K19" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="L19" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="M19" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="N19" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="O19" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="P19" s="1" t="s">
+        <v>35</v>
+      </c>
+      <c r="Q19" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="R19" s="1" t="s">
+        <v>37</v>
+      </c>
+      <c r="S19" s="1" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="20" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A20" s="3" t="s">
+        <v>28</v>
+      </c>
+      <c r="B20" s="3" t="s">
+        <v>16</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="G20" s="3" t="s">
+        <v>3</v>
+      </c>
+      <c r="H20" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="B6" s="7">
+      <c r="I20" s="3" t="s">
+        <v>5</v>
+      </c>
+      <c r="J20" s="3" t="s">
+        <v>6</v>
+      </c>
+      <c r="K20" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="L20" s="3" t="s">
+        <v>8</v>
+      </c>
+      <c r="M20" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="N20" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="C6" s="5"/>
-      <c r="D6" s="10">
-        <v>4</v>
-      </c>
-      <c r="E6" s="11">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A7" s="6">
-        <v>5</v>
-      </c>
-      <c r="B7" s="7">
+      <c r="O20" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="C7" s="5"/>
-      <c r="D7" s="10">
-        <v>5</v>
-      </c>
-      <c r="E7" s="11">
-        <v>11</v>
-      </c>
-    </row>
-    <row r="8" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A8" s="8">
-        <v>6</v>
-      </c>
-      <c r="B8" s="9"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="12">
-        <v>6</v>
-      </c>
-      <c r="E8" s="13"/>
-    </row>
-    <row r="9" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A9" s="5"/>
-    </row>
-    <row r="10" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A10" s="15" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="11" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A11" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="B11" s="1" t="s">
+      <c r="P20" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="Q20" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="R20" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="S20" s="3" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="21" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="A21" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="B21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="D21" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="C11" s="1" t="s">
+      <c r="E21" s="2" t="s">
         <v>19</v>
       </c>
-      <c r="D11" s="1" t="s">
+      <c r="F21" s="2" t="s">
         <v>20</v>
       </c>
-      <c r="E11" s="1" t="s">
+      <c r="G21" s="2" t="s">
         <v>21</v>
       </c>
-      <c r="F11" s="1" t="s">
+      <c r="H21" s="2" t="s">
         <v>22</v>
       </c>
-      <c r="G11" s="1" t="s">
+      <c r="I21" s="2" t="s">
         <v>23</v>
       </c>
-      <c r="H11" s="1" t="s">
+      <c r="J21" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="I11" s="1" t="s">
+      <c r="K21" s="2" t="s">
         <v>25</v>
       </c>
-      <c r="J11" s="1" t="s">
+      <c r="L21" s="2" t="s">
         <v>26</v>
       </c>
-      <c r="K11" s="1" t="s">
+      <c r="M21" s="2" t="s">
         <v>30</v>
       </c>
-      <c r="L11" s="1" t="s">
+      <c r="N21" s="2" t="s">
         <v>31</v>
       </c>
-      <c r="M11" s="1" t="s">
+      <c r="O21" s="2" t="s">
         <v>32</v>
       </c>
-      <c r="N11" s="1" t="s">
+      <c r="P21" s="2" t="s">
         <v>33</v>
       </c>
-      <c r="O11" s="1" t="s">
+      <c r="Q21" s="2" t="s">
         <v>34</v>
       </c>
-      <c r="P11" s="1" t="s">
+      <c r="R21" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="Q11" s="1" t="s">
+      <c r="S21" s="2" t="s">
         <v>36</v>
       </c>
-      <c r="R11" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="S11" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="12" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A12" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="C12" s="3" t="s">
-        <v>17</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="E12" s="3" t="s">
-        <v>1</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>2</v>
-      </c>
-      <c r="G12" s="3" t="s">
-        <v>3</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>4</v>
-      </c>
-      <c r="I12" s="3" t="s">
-        <v>5</v>
-      </c>
-      <c r="J12" s="3" t="s">
-        <v>6</v>
-      </c>
-      <c r="K12" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="L12" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="M12" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="N12" s="3" t="s">
-        <v>10</v>
-      </c>
-      <c r="O12" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="P12" s="3" t="s">
-        <v>12</v>
-      </c>
-      <c r="Q12" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="R12" s="3" t="s">
-        <v>14</v>
-      </c>
-      <c r="S12" s="3" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="13" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="A13" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="B13" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="C13" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="D13" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="E13" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F13" s="2" t="s">
-        <v>20</v>
-      </c>
-      <c r="G13" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="I13" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="J13" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="K13" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="L13" s="2" t="s">
-        <v>26</v>
-      </c>
-      <c r="M13" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="N13" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="O13" s="2" t="s">
-        <v>32</v>
-      </c>
-      <c r="P13" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="Q13" s="2" t="s">
-        <v>34</v>
-      </c>
-      <c r="R13" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="S13" s="2" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="14" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="D14" s="4" t="s">
+    </row>
+    <row r="22" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D22" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="4" t="s">
+      <c r="E22" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="F14" s="4" t="s">
+      <c r="F22" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="G14" s="4" t="s">
+      <c r="G22" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="H14" s="4" t="s">
+      <c r="H22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="I14" s="4" t="s">
+      <c r="I22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="J14" s="4" t="s">
+      <c r="J22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="K14" s="4" t="s">
+      <c r="K22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="L14" s="4" t="s">
+      <c r="L22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="M14" s="4" t="s">
+      <c r="M22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="N14" s="4" t="s">
+      <c r="N22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="O14" s="4" t="s">
+      <c r="O22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="P14" s="4" t="s">
+      <c r="P22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="Q14" s="4" t="s">
+      <c r="Q22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="R14" s="4" t="s">
+      <c r="R22" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="S14" s="4" t="s">
+      <c r="S22" s="4" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="15" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="D15" t="s">
+    <row r="23" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D23" t="s">
         <v>46</v>
       </c>
-      <c r="E15" t="s">
+      <c r="E23" t="s">
         <v>56</v>
       </c>
-      <c r="F15" t="s">
+      <c r="F23" t="s">
         <v>67</v>
       </c>
-      <c r="G15" t="s">
+      <c r="G23" t="s">
         <v>78</v>
       </c>
-      <c r="H15" s="14" t="s">
+      <c r="H23" s="6" t="s">
         <v>100</v>
       </c>
-      <c r="I15" t="s">
+      <c r="I23" t="s">
         <v>105</v>
       </c>
-      <c r="J15" t="s">
+      <c r="J23" t="s">
         <v>110</v>
       </c>
-      <c r="K15" t="s">
+      <c r="K23" t="s">
         <v>115</v>
       </c>
-      <c r="L15" t="s">
+      <c r="L23" t="s">
         <v>120</v>
       </c>
-      <c r="M15" t="s">
+      <c r="M23" t="s">
         <v>125</v>
       </c>
-      <c r="N15" t="s">
+      <c r="N23" t="s">
         <v>130</v>
       </c>
-      <c r="O15" t="s">
+      <c r="O23" t="s">
         <v>135</v>
       </c>
-      <c r="P15" t="s">
+      <c r="P23" t="s">
         <v>140</v>
       </c>
-      <c r="Q15" t="s">
+      <c r="Q23" t="s">
         <v>145</v>
       </c>
-      <c r="R15" t="s">
+      <c r="R23" t="s">
         <v>150</v>
       </c>
     </row>
-    <row r="16" spans="1:19" x14ac:dyDescent="0.45">
-      <c r="D16" t="s">
+    <row r="24" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D24" t="s">
         <v>47</v>
       </c>
-      <c r="E16" t="s">
+      <c r="E24" t="s">
         <v>57</v>
       </c>
-      <c r="F16" t="s">
+      <c r="F24" t="s">
         <v>68</v>
       </c>
-      <c r="G16" t="s">
+      <c r="G24" t="s">
         <v>79</v>
       </c>
-      <c r="H16" s="14" t="s">
+      <c r="H24" s="6" t="s">
         <v>101</v>
       </c>
-      <c r="I16" t="s">
+      <c r="I24" t="s">
         <v>106</v>
       </c>
-      <c r="J16" t="s">
+      <c r="J24" t="s">
         <v>111</v>
       </c>
-      <c r="K16" t="s">
+      <c r="K24" t="s">
         <v>116</v>
       </c>
-      <c r="L16" t="s">
+      <c r="L24" t="s">
         <v>121</v>
       </c>
-      <c r="M16" t="s">
+      <c r="M24" t="s">
         <v>126</v>
       </c>
-      <c r="N16" t="s">
+      <c r="N24" t="s">
         <v>131</v>
       </c>
-      <c r="O16" t="s">
+      <c r="O24" t="s">
         <v>136</v>
       </c>
-      <c r="P16" t="s">
+      <c r="P24" t="s">
         <v>141</v>
       </c>
-      <c r="Q16" t="s">
+      <c r="Q24" t="s">
         <v>146</v>
       </c>
-      <c r="R16" t="s">
+      <c r="R24" t="s">
         <v>151</v>
       </c>
     </row>
-    <row r="17" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D17" t="s">
+    <row r="25" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D25" t="s">
         <v>48</v>
       </c>
-      <c r="E17" t="s">
+      <c r="E25" t="s">
         <v>58</v>
       </c>
-      <c r="F17" t="s">
+      <c r="F25" t="s">
         <v>69</v>
       </c>
-      <c r="G17" t="s">
+      <c r="G25" t="s">
         <v>80</v>
       </c>
-      <c r="H17" s="14" t="s">
+      <c r="H25" s="6" t="s">
         <v>102</v>
       </c>
-      <c r="I17" t="s">
+      <c r="I25" t="s">
         <v>107</v>
       </c>
-      <c r="J17" t="s">
+      <c r="J25" t="s">
         <v>112</v>
       </c>
-      <c r="K17" t="s">
+      <c r="K25" t="s">
         <v>117</v>
       </c>
-      <c r="L17" t="s">
+      <c r="L25" t="s">
         <v>122</v>
       </c>
-      <c r="M17" t="s">
+      <c r="M25" t="s">
         <v>127</v>
       </c>
-      <c r="N17" t="s">
+      <c r="N25" t="s">
         <v>132</v>
       </c>
-      <c r="O17" t="s">
+      <c r="O25" t="s">
         <v>137</v>
       </c>
-      <c r="P17" t="s">
+      <c r="P25" t="s">
         <v>142</v>
       </c>
-      <c r="Q17" t="s">
+      <c r="Q25" t="s">
         <v>147</v>
       </c>
-      <c r="R17" t="s">
+      <c r="R25" t="s">
         <v>152</v>
       </c>
     </row>
-    <row r="18" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D18" t="s">
+    <row r="26" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D26" t="s">
         <v>49</v>
       </c>
-      <c r="E18" t="s">
+      <c r="E26" t="s">
         <v>59</v>
       </c>
-      <c r="F18" t="s">
+      <c r="F26" t="s">
         <v>70</v>
       </c>
-      <c r="G18" t="s">
+      <c r="G26" t="s">
         <v>81</v>
       </c>
-      <c r="H18" s="14" t="s">
+      <c r="H26" s="6" t="s">
         <v>103</v>
       </c>
-      <c r="I18" t="s">
+      <c r="I26" t="s">
         <v>108</v>
       </c>
-      <c r="J18" t="s">
+      <c r="J26" t="s">
         <v>113</v>
       </c>
-      <c r="K18" t="s">
+      <c r="K26" t="s">
         <v>118</v>
       </c>
-      <c r="L18" t="s">
+      <c r="L26" t="s">
         <v>123</v>
       </c>
-      <c r="M18" t="s">
+      <c r="M26" t="s">
         <v>128</v>
       </c>
-      <c r="N18" t="s">
+      <c r="N26" t="s">
         <v>133</v>
       </c>
-      <c r="O18" t="s">
+      <c r="O26" t="s">
         <v>138</v>
       </c>
-      <c r="P18" t="s">
+      <c r="P26" t="s">
         <v>143</v>
       </c>
-      <c r="Q18" t="s">
+      <c r="Q26" t="s">
         <v>148</v>
       </c>
-      <c r="R18" t="s">
+      <c r="R26" t="s">
         <v>153</v>
       </c>
     </row>
-    <row r="19" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D19" t="s">
+    <row r="27" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D27" t="s">
         <v>50</v>
       </c>
-      <c r="E19" t="s">
+      <c r="E27" t="s">
         <v>60</v>
       </c>
-      <c r="F19" t="s">
+      <c r="F27" t="s">
         <v>71</v>
       </c>
-      <c r="G19" t="s">
+      <c r="G27" t="s">
         <v>82</v>
       </c>
-      <c r="H19" s="14" t="s">
+      <c r="H27" s="6" t="s">
         <v>93</v>
       </c>
-      <c r="I19" t="s">
+      <c r="I27" t="s">
         <v>98</v>
       </c>
-      <c r="J19" t="s">
+      <c r="J27" t="s">
         <v>94</v>
       </c>
-      <c r="K19" t="s">
+      <c r="K27" t="s">
         <v>99</v>
       </c>
-      <c r="L19" t="s">
+      <c r="L27" t="s">
         <v>95</v>
       </c>
-      <c r="M19" t="s">
+      <c r="M27" t="s">
         <v>89</v>
       </c>
-      <c r="N19" t="s">
+      <c r="N27" t="s">
         <v>96</v>
       </c>
-      <c r="O19" t="s">
+      <c r="O27" t="s">
         <v>90</v>
       </c>
-      <c r="P19" t="s">
+      <c r="P27" t="s">
         <v>97</v>
       </c>
-      <c r="Q19" t="s">
+      <c r="Q27" t="s">
         <v>91</v>
       </c>
-      <c r="R19" t="s">
+      <c r="R27" t="s">
         <v>92</v>
       </c>
     </row>
-    <row r="20" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D20" t="s">
+    <row r="28" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D28" t="s">
         <v>51</v>
       </c>
-      <c r="E20" t="s">
+      <c r="E28" t="s">
         <v>61</v>
       </c>
-      <c r="F20" t="s">
+      <c r="F28" t="s">
         <v>72</v>
       </c>
-      <c r="G20" t="s">
+      <c r="G28" t="s">
         <v>83</v>
       </c>
-      <c r="H20" s="14" t="s">
+      <c r="H28" s="6" t="s">
         <v>104</v>
       </c>
-      <c r="I20" t="s">
+      <c r="I28" t="s">
         <v>109</v>
       </c>
-      <c r="J20" t="s">
+      <c r="J28" t="s">
         <v>114</v>
       </c>
-      <c r="K20" t="s">
+      <c r="K28" t="s">
         <v>119</v>
       </c>
-      <c r="L20" t="s">
+      <c r="L28" t="s">
         <v>124</v>
       </c>
-      <c r="M20" t="s">
+      <c r="M28" t="s">
         <v>129</v>
       </c>
-      <c r="N20" t="s">
+      <c r="N28" t="s">
         <v>134</v>
       </c>
-      <c r="O20" t="s">
+      <c r="O28" t="s">
         <v>139</v>
       </c>
-      <c r="P20" t="s">
+      <c r="P28" t="s">
         <v>144</v>
       </c>
-      <c r="Q20" t="s">
+      <c r="Q28" t="s">
         <v>149</v>
       </c>
-      <c r="R20" t="s">
+      <c r="R28" t="s">
         <v>154</v>
       </c>
     </row>
-    <row r="21" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D21" t="s">
+    <row r="29" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D29" t="s">
         <v>52</v>
       </c>
-      <c r="E21" t="s">
+      <c r="E29" t="s">
         <v>62</v>
       </c>
-      <c r="F21" t="s">
+      <c r="F29" t="s">
         <v>73</v>
       </c>
-      <c r="G21" t="s">
+      <c r="G29" t="s">
         <v>84</v>
       </c>
-      <c r="H21" s="14"/>
-    </row>
-    <row r="22" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D22" t="s">
+      <c r="H29" s="6"/>
+    </row>
+    <row r="30" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D30" t="s">
         <v>53</v>
       </c>
-      <c r="E22" t="s">
+      <c r="E30" t="s">
         <v>63</v>
       </c>
-      <c r="F22" t="s">
+      <c r="F30" t="s">
         <v>74</v>
       </c>
-      <c r="G22" t="s">
+      <c r="G30" t="s">
         <v>85</v>
       </c>
-      <c r="H22" s="14"/>
-    </row>
-    <row r="23" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D23" t="s">
+      <c r="H30" s="6"/>
+    </row>
+    <row r="31" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D31" t="s">
         <v>54</v>
       </c>
-      <c r="E23" t="s">
+      <c r="E31" t="s">
         <v>64</v>
       </c>
-      <c r="F23" t="s">
+      <c r="F31" t="s">
         <v>75</v>
       </c>
-      <c r="G23" t="s">
+      <c r="G31" t="s">
         <v>86</v>
       </c>
-      <c r="H23" s="14"/>
-    </row>
-    <row r="24" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D24" t="s">
+      <c r="H31" s="6"/>
+    </row>
+    <row r="32" spans="1:19" x14ac:dyDescent="0.45">
+      <c r="D32" t="s">
         <v>156</v>
       </c>
-      <c r="E24" t="s">
+      <c r="E32" t="s">
         <v>65</v>
       </c>
-      <c r="F24" t="s">
+      <c r="F32" t="s">
         <v>76</v>
       </c>
-      <c r="G24" t="s">
+      <c r="G32" t="s">
         <v>87</v>
       </c>
-      <c r="H24" s="14"/>
-    </row>
-    <row r="25" spans="4:18" x14ac:dyDescent="0.45">
-      <c r="D25" t="s">
+      <c r="H32" s="6"/>
+    </row>
+    <row r="33" spans="4:8" x14ac:dyDescent="0.45">
+      <c r="D33" t="s">
         <v>55</v>
       </c>
-      <c r="E25" t="s">
+      <c r="E33" t="s">
         <v>66</v>
       </c>
-      <c r="F25" t="s">
+      <c r="F33" t="s">
         <v>77</v>
       </c>
-      <c r="G25" t="s">
+      <c r="G33" t="s">
         <v>88</v>
       </c>
-      <c r="H25" s="14"/>
+      <c r="H33" s="6"/>
     </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A1:B1"/>
-    <mergeCell ref="D1:E1"/>
-    <mergeCell ref="A2:B2"/>
-    <mergeCell ref="D2:E2"/>
-  </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>